<commit_message>
fix: restore 15s timeout and harden runtime tick timing
</commit_message>
<xml_diff>
--- a/docs/design/蛋仔--大富翁--常量表.xlsx
+++ b/docs/design/蛋仔--大富翁--常量表.xlsx
@@ -415,94 +415,94 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="3" max="3" width="15.875" customWidth="1"/>
-    <col min="4" max="4" width="26" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="1">
-        <v>1</v>
-      </c>
-      <c r="B3" s="2">
-        <v>100000</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D3" s="2"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="1">
-        <v>2</v>
-      </c>
-      <c r="B4" s="2">
-        <v>1</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="1">
-        <v>3</v>
-      </c>
-      <c r="B5" s="2">
-        <v>2</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D5" s="2"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6" s="1">
-        <v>4</v>
-      </c>
-      <c r="B6" s="2">
-        <v>10</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6" s="2"/>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
+<ns0:worksheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0000-000000000000}">
+  <ns0:dimension ref="A1:D6"/>
+  <ns0:sheetFormatPr defaultRowHeight="14.25" ns3:dyDescent="0.2"/>
+  <ns0:cols>
+    <ns0:col min="3" max="3" width="15.875" customWidth="1"/>
+    <ns0:col min="4" max="4" width="26" customWidth="1"/>
+  </ns0:cols>
+  <ns0:sheetData>
+    <ns0:row r="1" spans="1:4" ns3:dyDescent="0.2">
+      <ns0:c r="A1" s="1" t="s">
+        <ns0:v>2</ns0:v>
+      </ns0:c>
+      <ns0:c r="B1" s="1" t="s">
+        <ns0:v>3</ns0:v>
+      </ns0:c>
+      <ns0:c r="C1" s="1" t="s">
+        <ns0:v>4</ns0:v>
+      </ns0:c>
+      <ns0:c r="D1" s="1" t="s">
+        <ns0:v>5</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="2" spans="1:4" ns3:dyDescent="0.2">
+      <ns0:c r="A2" s="1" t="s">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="B2" s="1" t="s">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="C2" s="1" t="s">
+        <ns0:v>1</ns0:v>
+      </ns0:c>
+      <ns0:c r="D2" s="1" t="s">
+        <ns0:v>1</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="3" spans="1:4" ns3:dyDescent="0.2">
+      <ns0:c r="A3" s="1">
+        <ns0:v>1</ns0:v>
+      </ns0:c>
+      <ns0:c r="B3" s="2">
+        <ns0:v>100000</ns0:v>
+      </ns0:c>
+      <ns0:c r="C3" s="2" t="s">
+        <ns0:v>6</ns0:v>
+      </ns0:c>
+      <ns0:c r="D3" s="2"/>
+    </ns0:row>
+    <ns0:row r="4" spans="1:4" ns3:dyDescent="0.2">
+      <ns0:c r="A4" s="1">
+        <ns0:v>2</ns0:v>
+      </ns0:c>
+      <ns0:c r="B4" s="2">
+        <ns0:v>1</ns0:v>
+      </ns0:c>
+      <ns0:c r="C4" s="2" t="s">
+        <ns0:v>7</ns0:v>
+      </ns0:c>
+      <ns0:c r="D4" s="2" t="s">
+        <ns0:v>8</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="5" spans="1:4" ns3:dyDescent="0.2">
+      <ns0:c r="A5" s="1">
+        <ns0:v>3</ns0:v>
+      </ns0:c>
+      <ns0:c r="B5" s="2">
+        <ns0:v>2</ns0:v>
+      </ns0:c>
+      <ns0:c r="C5" s="2" t="s">
+        <ns0:v>9</ns0:v>
+      </ns0:c>
+      <ns0:c r="D5" s="2"/>
+    </ns0:row>
+    <ns0:row r="6" spans="1:4" ns3:dyDescent="0.2">
+      <ns0:c r="A6" s="1">
+        <ns0:v>4</ns0:v>
+      </ns0:c>
+      <ns0:c r="B6" s="2">
+        <ns0:v>15</ns0:v>
+      </ns0:c>
+      <ns0:c r="C6" s="2" t="s">
+        <ns0:v>10</ns0:v>
+      </ns0:c>
+      <ns0:c r="D6" s="2"/>
+    </ns0:row>
+  </ns0:sheetData>
+  <ns0:phoneticPr fontId="1" type="noConversion"/>
+  <ns0:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</ns0:worksheet>
 </file>
</xml_diff>

<commit_message>
fix(ui): unify avatar sizing and stabilize release-trimmed regression
- switch base panel player avatar to native_size strategy

- capture player colors from base panel floor nodes with fallback

- add regression mode auto/dev/release_trimmed with temporary filtered cases

- relax forced_move sanity check to destination validity

- refresh generated config and design sheets
</commit_message>
<xml_diff>
--- a/docs/design/蛋仔--大富翁--常量表.xlsx
+++ b/docs/design/蛋仔--大富翁--常量表.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\策划文档\大富翁\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lzx_8\Desktop\eggitor\1_开发中\大富翁\策划案\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11AA718F-FB7E-4A7D-AAF4-9B785F55D1AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A442E821-4695-4DF7-8D0E-4C98E83DB79E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -75,17 +75,17 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -415,94 +415,94 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<ns0:worksheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0000-000000000000}">
-  <ns0:dimension ref="A1:D6"/>
-  <ns0:sheetFormatPr defaultRowHeight="14.25" ns3:dyDescent="0.2"/>
-  <ns0:cols>
-    <ns0:col min="3" max="3" width="15.875" customWidth="1"/>
-    <ns0:col min="4" max="4" width="26" customWidth="1"/>
-  </ns0:cols>
-  <ns0:sheetData>
-    <ns0:row r="1" spans="1:4" ns3:dyDescent="0.2">
-      <ns0:c r="A1" s="1" t="s">
-        <ns0:v>2</ns0:v>
-      </ns0:c>
-      <ns0:c r="B1" s="1" t="s">
-        <ns0:v>3</ns0:v>
-      </ns0:c>
-      <ns0:c r="C1" s="1" t="s">
-        <ns0:v>4</ns0:v>
-      </ns0:c>
-      <ns0:c r="D1" s="1" t="s">
-        <ns0:v>5</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="2" spans="1:4" ns3:dyDescent="0.2">
-      <ns0:c r="A2" s="1" t="s">
-        <ns0:v>0</ns0:v>
-      </ns0:c>
-      <ns0:c r="B2" s="1" t="s">
-        <ns0:v>0</ns0:v>
-      </ns0:c>
-      <ns0:c r="C2" s="1" t="s">
-        <ns0:v>1</ns0:v>
-      </ns0:c>
-      <ns0:c r="D2" s="1" t="s">
-        <ns0:v>1</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="3" spans="1:4" ns3:dyDescent="0.2">
-      <ns0:c r="A3" s="1">
-        <ns0:v>1</ns0:v>
-      </ns0:c>
-      <ns0:c r="B3" s="2">
-        <ns0:v>100000</ns0:v>
-      </ns0:c>
-      <ns0:c r="C3" s="2" t="s">
-        <ns0:v>6</ns0:v>
-      </ns0:c>
-      <ns0:c r="D3" s="2"/>
-    </ns0:row>
-    <ns0:row r="4" spans="1:4" ns3:dyDescent="0.2">
-      <ns0:c r="A4" s="1">
-        <ns0:v>2</ns0:v>
-      </ns0:c>
-      <ns0:c r="B4" s="2">
-        <ns0:v>1</ns0:v>
-      </ns0:c>
-      <ns0:c r="C4" s="2" t="s">
-        <ns0:v>7</ns0:v>
-      </ns0:c>
-      <ns0:c r="D4" s="2" t="s">
-        <ns0:v>8</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="5" spans="1:4" ns3:dyDescent="0.2">
-      <ns0:c r="A5" s="1">
-        <ns0:v>3</ns0:v>
-      </ns0:c>
-      <ns0:c r="B5" s="2">
-        <ns0:v>2</ns0:v>
-      </ns0:c>
-      <ns0:c r="C5" s="2" t="s">
-        <ns0:v>9</ns0:v>
-      </ns0:c>
-      <ns0:c r="D5" s="2"/>
-    </ns0:row>
-    <ns0:row r="6" spans="1:4" ns3:dyDescent="0.2">
-      <ns0:c r="A6" s="1">
-        <ns0:v>4</ns0:v>
-      </ns0:c>
-      <ns0:c r="B6" s="2">
-        <ns0:v>15</ns0:v>
-      </ns0:c>
-      <ns0:c r="C6" s="2" t="s">
-        <ns0:v>10</ns0:v>
-      </ns0:c>
-      <ns0:c r="D6" s="2"/>
-    </ns0:row>
-  </ns0:sheetData>
-  <ns0:phoneticPr fontId="1" type="noConversion"/>
-  <ns0:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</ns0:worksheet>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="3" max="3" width="15.85546875" customWidth="1"/>
+    <col min="4" max="4" width="26" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="1">
+        <v>1</v>
+      </c>
+      <c r="B3" s="2">
+        <v>100000</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" s="2"/>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="1">
+        <v>2</v>
+      </c>
+      <c r="B4" s="2">
+        <v>1</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="1">
+        <v>3</v>
+      </c>
+      <c r="B5" s="2">
+        <v>2</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="2"/>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" s="1">
+        <v>4</v>
+      </c>
+      <c r="B6" s="2">
+        <v>15</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="2"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>